<commit_message>
08/06/2026, CC: created a draft mod to batch invalidate files and modified main app to account for it
</commit_message>
<xml_diff>
--- a/inst/extdata/data_flag_template.xlsx
+++ b/inst/extdata/data_flag_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cehacuk-my.sharepoint.com/personal/jamcas_ceh_ac_uk/Documents/MetQC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cehacuk-my.sharepoint.com/personal/clacap_ceh_ac_uk/Documents/metamet/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{08C4B469-E65D-4754-97D9-E747AEE8A36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{08C4B469-E65D-4754-97D9-E747AEE8A36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DF9231F-1554-479B-BFF3-14845664775E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="403" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8210" yWindow="1860" windowWidth="14400" windowHeight="8170" tabRatio="403" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Weekly checksheet" sheetId="1" r:id="rId1"/>
@@ -1253,15 +1253,6 @@
     <t>start_time</t>
   </si>
   <si>
-    <t>End_time</t>
-  </si>
-  <si>
-    <t>QC variable name</t>
-  </si>
-  <si>
-    <t>Comment</t>
-  </si>
-  <si>
     <t>list of names drop down</t>
   </si>
   <si>
@@ -1275,6 +1266,15 @@
   </si>
   <si>
     <t>QC_name</t>
+  </si>
+  <si>
+    <t>end_time</t>
+  </si>
+  <si>
+    <t>QC_variable_name</t>
+  </si>
+  <si>
+    <t>comment</t>
   </si>
 </sst>
 </file>
@@ -2116,16 +2116,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I191"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1"/>
   <cols>
     <col min="1" max="1" width="59" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" customWidth="1"/>
-    <col min="6" max="6" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" customWidth="1"/>
+    <col min="3" max="3" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.7265625" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" customWidth="1"/>
+    <col min="6" max="6" width="3.453125" customWidth="1"/>
     <col min="7" max="9" width="0" hidden="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" hidden="1"/>
+    <col min="10" max="16384" width="9.1796875" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -2133,8 +2133,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.75" thickBot="1"/>
-    <row r="3" spans="1:6" ht="15.75" thickBot="1">
+    <row r="2" spans="1:6" ht="15" thickBot="1"/>
+    <row r="3" spans="1:6" ht="15" thickBot="1">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>46169</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75" thickBot="1">
+    <row r="4" spans="1:6" ht="15" thickBot="1">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2150,7 +2150,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.75" thickBot="1">
+    <row r="5" spans="1:6" ht="15" thickBot="1">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.75" thickBot="1">
+    <row r="6" spans="1:6" ht="15" thickBot="1">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -2179,7 +2179,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.75" thickBot="1">
+    <row r="9" spans="1:6" ht="15" thickBot="1">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -2187,7 +2187,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15.75" thickBot="1">
+    <row r="10" spans="1:6" ht="15" thickBot="1">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -2201,7 +2201,7 @@
         <v>14.13</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15.75" thickBot="1">
+    <row r="11" spans="1:6" ht="15" thickBot="1">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -2213,10 +2213,10 @@
       </c>
       <c r="E11" s="11"/>
     </row>
-    <row r="12" spans="1:6" ht="15.75" thickBot="1">
+    <row r="12" spans="1:6" ht="15" thickBot="1">
       <c r="B12" s="3"/>
     </row>
-    <row r="13" spans="1:6" ht="15.75" thickBot="1">
+    <row r="13" spans="1:6" ht="15" thickBot="1">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -2227,7 +2227,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15.75" thickBot="1">
+    <row r="14" spans="1:6" ht="15" thickBot="1">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -2241,7 +2241,7 @@
         <v>13.87</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.75" thickBot="1">
+    <row r="15" spans="1:6" ht="15" thickBot="1">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2256,12 +2256,12 @@
       </c>
     </row>
     <row r="16" spans="1:6"/>
-    <row r="17" spans="1:5" ht="15.75" thickBot="1">
+    <row r="17" spans="1:5" ht="15" thickBot="1">
       <c r="A17" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15.75" thickBot="1">
+    <row r="18" spans="1:5" ht="15" thickBot="1">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="15.75" thickBot="1">
+    <row r="19" spans="1:5" ht="15" thickBot="1">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>13.62</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15.75" thickBot="1">
+    <row r="20" spans="1:5" ht="15" thickBot="1">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -2301,7 +2301,7 @@
       </c>
     </row>
     <row r="21" spans="1:5"/>
-    <row r="22" spans="1:5" ht="15.75" thickBot="1">
+    <row r="22" spans="1:5" ht="15" thickBot="1">
       <c r="A22" s="1" t="s">
         <v>27</v>
       </c>
@@ -2309,7 +2309,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="19.5" thickBot="1">
+    <row r="23" spans="1:5" ht="18" thickBot="1">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -2323,7 +2323,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="15.75" thickBot="1">
+    <row r="24" spans="1:5" ht="15" thickBot="1">
       <c r="A24" t="s">
         <v>31</v>
       </c>
@@ -2337,7 +2337,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="15.75" thickBot="1">
+    <row r="25" spans="1:5" ht="15" thickBot="1">
       <c r="A25" t="s">
         <v>33</v>
       </c>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="D25" s="4"/>
     </row>
-    <row r="26" spans="1:5" ht="15.75" thickBot="1">
+    <row r="26" spans="1:5" ht="15" thickBot="1">
       <c r="A26" t="s">
         <v>34</v>
       </c>
@@ -2364,7 +2364,7 @@
       </c>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" ht="15.75" thickBot="1">
+    <row r="28" spans="1:5" ht="15" thickBot="1">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="E28" s="3"/>
     </row>
-    <row r="29" spans="1:5" ht="15.75" thickBot="1">
+    <row r="29" spans="1:5" ht="15" thickBot="1">
       <c r="A29" t="s">
         <v>13</v>
       </c>
@@ -2381,12 +2381,12 @@
         <v>12.77</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15.75" thickBot="1">
+    <row r="30" spans="1:5" ht="15" thickBot="1">
       <c r="D30" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="15.75" thickBot="1">
+    <row r="31" spans="1:5" ht="15" thickBot="1">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -2397,7 +2397,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="15.75" thickBot="1">
+    <row r="32" spans="1:5" ht="15" thickBot="1">
       <c r="A32" t="s">
         <v>39</v>
       </c>
@@ -2411,7 +2411,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="15.75" thickBot="1">
+    <row r="33" spans="1:6" ht="15" thickBot="1">
       <c r="A33" t="s">
         <v>41</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="15.75" thickBot="1">
+    <row r="34" spans="1:6" ht="15" thickBot="1">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -2430,7 +2430,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="15.75" thickBot="1">
+    <row r="35" spans="1:6" ht="15" thickBot="1">
       <c r="D35" s="6" t="s">
         <v>44</v>
       </c>
@@ -2438,7 +2438,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="15.75" thickBot="1">
+    <row r="36" spans="1:6" ht="15" thickBot="1">
       <c r="A36" s="1" t="s">
         <v>45</v>
       </c>
@@ -2449,7 +2449,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="15.75" thickBot="1">
+    <row r="37" spans="1:6" ht="15" thickBot="1">
       <c r="A37" t="s">
         <v>47</v>
       </c>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="D37" s="7"/>
     </row>
-    <row r="38" spans="1:6" ht="15.75" thickBot="1">
+    <row r="38" spans="1:6" ht="15" thickBot="1">
       <c r="A38" t="s">
         <v>48</v>
       </c>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D38" s="7"/>
     </row>
-    <row r="39" spans="1:6" ht="15.75" thickBot="1">
+    <row r="39" spans="1:6" ht="15" thickBot="1">
       <c r="A39" t="s">
         <v>49</v>
       </c>
@@ -2490,7 +2490,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="15.75" thickBot="1">
+    <row r="43" spans="1:6" ht="15" thickBot="1">
       <c r="A43" s="1" t="s">
         <v>51</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="15.75" thickBot="1">
+    <row r="44" spans="1:6" ht="15" thickBot="1">
       <c r="A44" t="s">
         <v>53</v>
       </c>
@@ -2512,7 +2512,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="15.75" thickBot="1">
+    <row r="45" spans="1:6" ht="15" thickBot="1">
       <c r="A45" t="s">
         <v>56</v>
       </c>
@@ -2526,7 +2526,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="15.75" thickBot="1">
+    <row r="46" spans="1:6" ht="15" thickBot="1">
       <c r="A46" t="s">
         <v>58</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>35.47</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="15.75" thickBot="1">
+    <row r="47" spans="1:6" ht="15" thickBot="1">
       <c r="A47" t="s">
         <v>60</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>25.14</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="15.75" thickBot="1">
+    <row r="48" spans="1:6" ht="15" thickBot="1">
       <c r="A48" t="s">
         <v>62</v>
       </c>
@@ -2568,7 +2568,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="15.75" thickBot="1">
+    <row r="49" spans="1:5" ht="15" thickBot="1">
       <c r="A49" t="s">
         <v>64</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="15.75" thickBot="1">
+    <row r="50" spans="1:5" ht="15" thickBot="1">
       <c r="A50" s="19" t="s">
         <v>66</v>
       </c>
@@ -2592,12 +2592,12 @@
       <c r="D50" s="7"/>
       <c r="E50" s="1"/>
     </row>
-    <row r="51" spans="1:5" ht="15.75" thickBot="1">
+    <row r="51" spans="1:5" ht="15" thickBot="1">
       <c r="D51" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="15.75" thickBot="1">
+    <row r="52" spans="1:5" ht="15" thickBot="1">
       <c r="A52" s="5" t="s">
         <v>68</v>
       </c>
@@ -2608,7 +2608,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="15.75" thickBot="1">
+    <row r="53" spans="1:5" ht="15" thickBot="1">
       <c r="A53" t="s">
         <v>53</v>
       </c>
@@ -2622,7 +2622,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="15.75" thickBot="1">
+    <row r="54" spans="1:5" ht="15" thickBot="1">
       <c r="A54" t="s">
         <v>71</v>
       </c>
@@ -2636,7 +2636,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="15.75" thickBot="1">
+    <row r="55" spans="1:5" ht="15" thickBot="1">
       <c r="A55" t="s">
         <v>73</v>
       </c>
@@ -2650,7 +2650,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="15.75" thickBot="1">
+    <row r="56" spans="1:5" ht="15" thickBot="1">
       <c r="A56" t="s">
         <v>60</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="15.75" thickBot="1">
+    <row r="57" spans="1:5" ht="15" thickBot="1">
       <c r="A57" t="s">
         <v>62</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="15.75" thickBot="1">
+    <row r="58" spans="1:5" ht="15" thickBot="1">
       <c r="A58" t="s">
         <v>77</v>
       </c>
@@ -2686,12 +2686,12 @@
         <v>3967.2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="15.75" thickBot="1">
+    <row r="59" spans="1:5" ht="15" thickBot="1">
       <c r="D59" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="15.75" thickBot="1">
+    <row r="60" spans="1:5" ht="15" thickBot="1">
       <c r="A60" s="1" t="s">
         <v>79</v>
       </c>
@@ -2702,7 +2702,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="15.75" thickBot="1">
+    <row r="61" spans="1:5" ht="15" thickBot="1">
       <c r="A61" t="s">
         <v>53</v>
       </c>
@@ -2716,7 +2716,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="15.75" thickBot="1">
+    <row r="62" spans="1:5" ht="15" thickBot="1">
       <c r="A62" t="s">
         <v>83</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="15.75" thickBot="1">
+    <row r="63" spans="1:5" ht="15" thickBot="1">
       <c r="A63" t="s">
         <v>84</v>
       </c>
@@ -2735,7 +2735,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="15.75" thickBot="1">
+    <row r="64" spans="1:5" ht="15" thickBot="1">
       <c r="D64" s="7" t="s">
         <v>86</v>
       </c>
@@ -2743,7 +2743,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="15.75" thickBot="1">
+    <row r="65" spans="1:6" ht="15" thickBot="1">
       <c r="A65" s="1" t="s">
         <v>87</v>
       </c>
@@ -2754,7 +2754,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="15.75" thickBot="1">
+    <row r="66" spans="1:6" ht="15" thickBot="1">
       <c r="A66" s="6" t="s">
         <v>89</v>
       </c>
@@ -2769,7 +2769,7 @@
       </c>
     </row>
     <row r="67" spans="1:6"/>
-    <row r="68" spans="1:6" ht="15.75" thickBot="1">
+    <row r="68" spans="1:6" ht="15" thickBot="1">
       <c r="A68" s="1" t="s">
         <v>91</v>
       </c>
@@ -2777,7 +2777,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="15.75" thickBot="1">
+    <row r="69" spans="1:6" ht="15" thickBot="1">
       <c r="A69" s="6" t="s">
         <v>93</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="15.75" thickBot="1">
+    <row r="70" spans="1:6" ht="15" thickBot="1">
       <c r="A70" s="6" t="s">
         <v>95</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="15.75" thickBot="1">
+    <row r="71" spans="1:6" ht="15" thickBot="1">
       <c r="A71" s="6" t="s">
         <v>97</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="15.75" thickBot="1">
+    <row r="72" spans="1:6" ht="15" thickBot="1">
       <c r="A72" s="7" t="s">
         <v>99</v>
       </c>
@@ -2833,12 +2833,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="73" spans="1:6" ht="15.75" thickBot="1">
+    <row r="73" spans="1:6" ht="15" thickBot="1">
       <c r="A73" s="16" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="15.75" thickBot="1">
+    <row r="74" spans="1:6" ht="15" thickBot="1">
       <c r="A74" s="6" t="s">
         <v>102</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="15.75" thickBot="1">
+    <row r="75" spans="1:6" ht="15" thickBot="1">
       <c r="A75" s="6" t="s">
         <v>104</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="76" spans="1:6" ht="15.75" thickBot="1">
+    <row r="76" spans="1:6" ht="15" thickBot="1">
       <c r="A76" s="6" t="s">
         <v>106</v>
       </c>
@@ -2891,12 +2891,12 @@
         <v>108</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="15.75" thickBot="1">
+    <row r="80" spans="1:6" ht="15" thickBot="1">
       <c r="D80" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="15.75" thickBot="1">
+    <row r="81" spans="1:6" ht="15" thickBot="1">
       <c r="A81" s="7" t="s">
         <v>110</v>
       </c>
@@ -2910,7 +2910,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="15.75" thickBot="1">
+    <row r="82" spans="1:6" ht="15" thickBot="1">
       <c r="A82" s="7" t="s">
         <v>113</v>
       </c>
@@ -2924,7 +2924,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="15.75" thickBot="1">
+    <row r="83" spans="1:6" ht="15" thickBot="1">
       <c r="A83" s="7" t="s">
         <v>115</v>
       </c>
@@ -2941,7 +2941,7 @@
     <row r="84" spans="1:6">
       <c r="D84" s="7"/>
     </row>
-    <row r="85" spans="1:6" ht="15.75" thickBot="1">
+    <row r="85" spans="1:6" ht="15" thickBot="1">
       <c r="A85" s="1" t="s">
         <v>117</v>
       </c>
@@ -2949,7 +2949,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="15.75" thickBot="1">
+    <row r="86" spans="1:6" ht="15" thickBot="1">
       <c r="A86" s="7" t="s">
         <v>119</v>
       </c>
@@ -2963,7 +2963,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="15.75" thickBot="1">
+    <row r="87" spans="1:6" ht="15" thickBot="1">
       <c r="A87" s="7" t="s">
         <v>121</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="15.75" thickBot="1">
+    <row r="88" spans="1:6" ht="15" thickBot="1">
       <c r="A88" s="7" t="s">
         <v>123</v>
       </c>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="D88" s="7"/>
     </row>
-    <row r="89" spans="1:6" ht="15.75" thickBot="1">
+    <row r="89" spans="1:6" ht="15" thickBot="1">
       <c r="A89" s="7" t="s">
         <v>124</v>
       </c>
@@ -2998,12 +2998,12 @@
     <row r="90" spans="1:6">
       <c r="D90" s="7"/>
     </row>
-    <row r="91" spans="1:6" ht="15.75" thickBot="1">
+    <row r="91" spans="1:6" ht="15" thickBot="1">
       <c r="A91" s="16" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="92" spans="1:6" ht="15.75" thickBot="1">
+    <row r="92" spans="1:6" ht="15" thickBot="1">
       <c r="A92" s="7" t="s">
         <v>126</v>
       </c>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="C92" s="7"/>
     </row>
-    <row r="93" spans="1:6" ht="15.75" thickBot="1">
+    <row r="93" spans="1:6" ht="15" thickBot="1">
       <c r="A93" s="7" t="s">
         <v>127</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="98" spans="1:5" ht="15.75" thickBot="1">
+    <row r="98" spans="1:5" ht="15" thickBot="1">
       <c r="A98" s="1" t="s">
         <v>129</v>
       </c>
@@ -3050,7 +3050,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="99" spans="1:5" ht="15.75" thickBot="1">
+    <row r="99" spans="1:5" ht="15" thickBot="1">
       <c r="A99" s="6" t="s">
         <v>131</v>
       </c>
@@ -3064,7 +3064,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="100" spans="1:5" ht="15.75" thickBot="1">
+    <row r="100" spans="1:5" ht="15" thickBot="1">
       <c r="A100" s="7" t="s">
         <v>133</v>
       </c>
@@ -3078,7 +3078,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="15.75" thickBot="1">
+    <row r="101" spans="1:5" ht="15" thickBot="1">
       <c r="A101" s="6" t="s">
         <v>134</v>
       </c>
@@ -3092,7 +3092,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="102" spans="1:5" ht="15.75" thickBot="1">
+    <row r="102" spans="1:5" ht="15" thickBot="1">
       <c r="A102" s="6" t="s">
         <v>136</v>
       </c>
@@ -3100,7 +3100,7 @@
         <v>270360</v>
       </c>
     </row>
-    <row r="103" spans="1:5" ht="15.75" thickBot="1">
+    <row r="103" spans="1:5" ht="15" thickBot="1">
       <c r="A103" s="6" t="s">
         <v>137</v>
       </c>
@@ -3109,7 +3109,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="15.75" thickBot="1">
+    <row r="104" spans="1:5" ht="15" thickBot="1">
       <c r="A104" s="7" t="s">
         <v>139</v>
       </c>
@@ -3122,7 +3122,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="105" spans="1:5" ht="15.75" thickBot="1">
+    <row r="105" spans="1:5" ht="15" thickBot="1">
       <c r="D105" s="7" t="s">
         <v>141</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="106" spans="1:5" ht="15.75" thickBot="1">
+    <row r="106" spans="1:5" ht="15" thickBot="1">
       <c r="A106" s="1" t="s">
         <v>142</v>
       </c>
@@ -3141,7 +3141,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="107" spans="1:5" ht="15.75" thickBot="1">
+    <row r="107" spans="1:5" ht="15" thickBot="1">
       <c r="A107" s="6" t="s">
         <v>144</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="108" spans="1:5" ht="15.75" thickBot="1">
+    <row r="108" spans="1:5" ht="15" thickBot="1">
       <c r="A108" s="7" t="s">
         <v>133</v>
       </c>
@@ -3163,12 +3163,12 @@
         <v>112</v>
       </c>
     </row>
-    <row r="109" spans="1:5" ht="15.75" thickBot="1">
+    <row r="109" spans="1:5" ht="15" thickBot="1">
       <c r="D109" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="110" spans="1:5" ht="15.75" thickBot="1">
+    <row r="110" spans="1:5" ht="15" thickBot="1">
       <c r="D110" s="7" t="s">
         <v>147</v>
       </c>
@@ -3177,7 +3177,7 @@
       </c>
     </row>
     <row r="111" spans="1:5"/>
-    <row r="112" spans="1:5" ht="15.75" thickBot="1">
+    <row r="112" spans="1:5" ht="15" thickBot="1">
       <c r="A112" s="2" t="s">
         <v>148</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="113" spans="1:5" ht="15.75" thickBot="1">
+    <row r="113" spans="1:5" ht="15" thickBot="1">
       <c r="A113" s="1" t="s">
         <v>150</v>
       </c>
@@ -3196,7 +3196,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="114" spans="1:5" ht="15.75" thickBot="1">
+    <row r="114" spans="1:5" ht="15" thickBot="1">
       <c r="A114" s="10" t="s">
         <v>152</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="115" spans="1:5" ht="15.75" thickBot="1">
+    <row r="115" spans="1:5" ht="15" thickBot="1">
       <c r="A115" s="10" t="s">
         <v>154</v>
       </c>
@@ -3220,7 +3220,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="116" spans="1:5" ht="26.25" thickBot="1">
+    <row r="116" spans="1:5" ht="25.5" thickBot="1">
       <c r="A116" s="10" t="s">
         <v>156</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="117" spans="1:5" ht="15.75" thickBot="1">
+    <row r="117" spans="1:5" ht="15" thickBot="1">
       <c r="A117" s="10" t="s">
         <v>158</v>
       </c>
@@ -3244,7 +3244,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="118" spans="1:5" ht="15.75" thickBot="1">
+    <row r="118" spans="1:5" ht="15" thickBot="1">
       <c r="A118" s="10" t="s">
         <v>160</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="119" spans="1:5" ht="15.75" thickBot="1">
+    <row r="119" spans="1:5" ht="15" thickBot="1">
       <c r="A119" s="14" t="s">
         <v>162</v>
       </c>
@@ -3268,7 +3268,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="120" spans="1:5" ht="15.75" thickBot="1">
+    <row r="120" spans="1:5" ht="15" thickBot="1">
       <c r="A120" s="14" t="s">
         <v>165</v>
       </c>
@@ -3280,7 +3280,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="121" spans="1:5" ht="15.75" thickBot="1">
+    <row r="121" spans="1:5" ht="15" thickBot="1">
       <c r="A121" s="10" t="s">
         <v>167</v>
       </c>
@@ -3294,7 +3294,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="122" spans="1:5" ht="15.75" thickBot="1">
+    <row r="122" spans="1:5" ht="15" thickBot="1">
       <c r="D122" s="10" t="s">
         <v>168</v>
       </c>
@@ -3302,12 +3302,12 @@
         <v>112</v>
       </c>
     </row>
-    <row r="123" spans="1:5" ht="15.75" thickBot="1">
+    <row r="123" spans="1:5" ht="15" thickBot="1">
       <c r="A123" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="124" spans="1:5" ht="15.75" thickBot="1">
+    <row r="124" spans="1:5" ht="15" thickBot="1">
       <c r="A124" s="10" t="s">
         <v>170</v>
       </c>
@@ -3316,7 +3316,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="125" spans="1:5" ht="15.75" thickBot="1">
+    <row r="125" spans="1:5" ht="15" thickBot="1">
       <c r="A125" s="10" t="s">
         <v>172</v>
       </c>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="E125" s="3"/>
     </row>
-    <row r="126" spans="1:5" ht="15.75" thickBot="1">
+    <row r="126" spans="1:5" ht="15" thickBot="1">
       <c r="A126" s="10" t="s">
         <v>174</v>
       </c>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="E126" s="3"/>
     </row>
-    <row r="127" spans="1:5" ht="15.75" thickBot="1">
+    <row r="127" spans="1:5" ht="15" thickBot="1">
       <c r="A127" s="10"/>
       <c r="D127" s="10"/>
       <c r="E127" s="3"/>
@@ -3403,8 +3403,8 @@
     <row r="148" spans="1:2"/>
     <row r="149" spans="1:2"/>
     <row r="150" spans="1:2"/>
-    <row r="151" spans="1:2" ht="15.75" thickBot="1"/>
-    <row r="152" spans="1:2" ht="15.75" thickBot="1">
+    <row r="151" spans="1:2" ht="15" thickBot="1"/>
+    <row r="152" spans="1:2" ht="15" thickBot="1">
       <c r="A152" s="6"/>
       <c r="B152" s="3"/>
     </row>
@@ -3537,7 +3537,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="B62:B63">
     <cfRule type="cellIs" dxfId="15" priority="23" operator="equal">
-      <formula>_xludf.N</formula>
+      <formula>N</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="14" priority="24" operator="lessThan">
       <formula>50</formula>
@@ -3629,12 +3629,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{536E7F24-1E64-4B6A-8ED0-D6A395E0881A}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -3642,22 +3642,22 @@
         <v>183</v>
       </c>
       <c r="B1" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C1" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D1" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="21"/>
       <c r="C2" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -3668,21 +3668,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6EA52BC-B6EA-4E7C-B805-7E4C2CAFBB1A}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B1" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C1" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>